<commit_message>
Weekly refresh Sep 7 2026: board verified at Fri Sep 4 close; PENG applied at 51.76 (+6.44%, second-sourced x2, was the one unconfirmed Sep-4 mover); QNT hi52/lo52 filled (86.79/46.54); SPCX & QNT listings independently re-verified - QNT removal patch stays unapplied; integrity audit: share counts clean (APH 2-for-1 expected), no stuck feeds, NASD/NYSE subtotals tie, groups consistent; FLAGGED: four Aug 5-7 fills (TSM/NVDA/CRM/ISRG) imply zero commission vs the flat 8.56 - needs POEMS contract notes; TOTALS investedEver identity drift now -9,210.82 (was -5,653.61) - semantics to pin; workbook rebuilt
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPmrZ7fsMLvtk7SU5XZAr4
</commit_message>
<xml_diff>
--- a/src/Pillar4_US_Portfolio_Workbook.xlsx
+++ b/src/Pillar4_US_Portfolio_Workbook.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sep 6, 2026 - WEEKLY REFRESH AND INTEGRITY AUDIT. The Sep 4 daily job reverted twelve &gt;=6% movers it could not second-source before its search budget ran out; this weekly run re-verified them. TEN CONFIRMED against a second independent dated source and applied at the Friday Sep 4 close with --allow, mcapB/pe/fpe/ps/peg rescaled by the exact price ratio per convention: SNDK 1,740.00 +11.90% (Google Finance 'Closed Sep 4, 4:00 PM GMT-4' agrees with stockanalysis to the cent), SKHY 177.00 +8.14% (GF + stockanalysis agree; the 24/7 Wall St intraday 174.38 was pre-close), BE 252.87 +7.35% (Motley Fool article of Sep 5 quotes 252.87 +17.32 exactly), KLAC 185.60 +7.32% (GF concurs, prev close ties to 172.94), IREN 44.68 +7.27% (GF dated close, +3.03 ties to the 41.65 board value), ADBE 266.51 -6.73% (24/7 Wall St Sep 4 CEO-succession piece quotes 266.51 -6.73% verbatim; GuruFocus concurs on a ~6-7% Friday fall), FPS 31.35 +6.56% off the Sep 2 close (Motley Fool at-close quote; GF intraday 31.44 at 11:29 AM concurs on level - accepted on the HNGE precedent, caveat recorded), SITM 612.09 +6.55% (Fool quote page shows 612.09 dated Sep 4 exactly, CAVEAT: its own day-change figure +1.07% implies a different Sep 3 close than the board's 574.47 - price corroborated, prior-day linkage not), NRG 119.02 +6.42% (GF dated close + Fool concur, open 111.29 ties to the board's 111.84 Sep 3 value), STX 849.28 +6.34% (GF dated close +50.67 ties exactly). ONE NOT CONFIRMED: PENG - GF still shows the Sep 3 close 48.63, Yahoo is stuck at Sep 1, CNN unusable; the pending 51.76 single-source print stays UNAPPLIED per the stale-beats-wrong rule and PENG remains at 48.63 with pxd 2026-09-03 showing honestly. Next daily run should confirm it. || AUDIT RESULTS, the checks the daily jobs cannot do. CLEAN: implied share counts (mcapB/price) moved &lt;1% on every name against the Aug 31 weekly build except APH, which doubled - the known 2-for-1 split applied in the Sep 4 POEMS reconciliation, correct; no ticker's price is stuck 7+ days (worst is PENG at 2 sessions); broker subtotals tie the Sep 4 POEMS screen to the cent - NASDAQ held cost 493,545.18 + NYSE 103,760.51 = 597,305.69; every fill since Jul 28 implies exactly the flat 8.56 POEMS commission (SKHY 8.57 / META 8.54 are fractional-share rounding); REALIZED, SOLD and MONTHLY byGroup are mutually consistent - July's byGroup ties byStock exactly under sale-time groups. FLAGGED, NOT FIXED: (1) NBIS realized gain is 1,404.52 in REALIZED but 1,404.51 in SOLD and MONTHLY - one cent, TOTALS ties to REALIZED; needs the POEMS figure to settle which. (2) Realized P&amp;L attributes to SALE-TIME groups: IREN g13, ORCL g10, SNPS g10, APP g10 predate the Aug 31 reclassification sweep (now g21/g13/g1/g19), so per-group realized figures reflect history, not today's grouping - semantics to be aware of, not corruption. (3) SNDK carries ath 1,804.00 BELOW hi52 2,354.39 and SITM ath 901.48 fractionally below hi52 901.81 - an all-time high cannot sit under a 52-week high unless ath means highest CLOSE and hi52 intraday; convention should be pinned and the two values re-sourced. (4) SNDK lo52 40.10 against a 1,740 price is a 43x 52-week range - plausible for the Feb-2025 spin-off in a memory supercycle but worth one look at POEMS. FIXED THIS RUN: the vestigial STOCKS.budget field had drifted from the authoritative POS budgets on 10 names (NVDA still showed 85,000 vs the 100,000 set Aug 27; FSLR, ONDS, IONQ, V, HUBB, AEP, SE, CAT, IREN showed None vs their 5,000 POS budgets) - synced to POS, which is what every page component actually reads, so nothing rendered changes. POS, TRADES, CASH, fundamentals untouched. IREN NOTE FOR THE SELLING TAB: the confirmed 44.68 close is 7.3% ABOVE the 41.65 carried on the IREN sell row; estimated proceeds there are now understated - no action taken, Salee executes. || Sep 5, 2026 - SELLING TAB ADDED at Salee's request as a control sheet for the liquidation programme. It carries, per name: shares, average cost, last close, target price or 'at market', estimated net proceeds, profit or loss, conviction, timing, the full reasoning, what happens to the budget after the sale, and a status of planned / placed / filled / cancelled. Estimated proceeds are net of the 8.56 flat POEMS commission - six sales cost 51.36 in total, which is why net proceeds are 14,110.13 against 14,161.49 gross, and net profit across the six is 711.69 rather than 763.05. || The sheet reads shares and cost live from the position book, so it cannot drift from the board, and falls back to stored values once a position is sold. A SELL DISCIPLINE panel records five standing rules, the first being: sell the thesis, not the price - three of the six are at a loss and one is up 112%, and that spread is deliberate. || ⚠️ THE TAB STATES PROMINENTLY THAT CLAUDE DOES NOT PLACE TRADES. Every row is an instruction for Salee to execute at POEMS; no position, cost or cash figure moves until he reports a fill. || Rows: TSLA and INTC at market (High conviction), ONDS at market with a limit if the spread is wide because the stock is thin (High), then IREN at 41.65, AAOI at 105.53 and QCOM at 168.74, all Medium and none urgent. || Build note: SELLBOOK was added to the CONSTS list in BOTH gen_dashboard.py and extract_data.py. A data block missing from either list is silently wiped on the next refresh. Verified by round-trip plus a headless Chromium render - no page errors, no horizontal overflow, all six reasoning blocks wrap without clipping. || Sep 5, 2026 - GPT-6 ASTRA ASSESSED (OpenAI, announced Sep 3). Salee asked whether it opens a new chapter for AI and who benefits. Five watch/decide rows added to this Schedule. || WHAT IT IS: a frontier model, not a new product category - 1,050,000 token context, 10 dollars in / 50 dollars out per million tokens (a 2.5x price rise), served on OpenAI's API, Azure and AWS Bedrock. The real advance is computer use: 72.6% on OSWorld in about 40 minutes per task versus 65.7% in about 75 minutes for the prior model. || ⚠️ THE 'STEP CHANGE' CLAIM IS CONTESTED AND SHOULD NOT BE TRADED AS FACT. Epoch AI ranked Astra first across 50+ tests; Artificial Analysis scored it flat versus its predecessor and BEHIND Anthropic's Claude Fable 5.1. OpenAI's headline 99.9% on ARC-AGI-3 was 62.7% when ARC Prize ran the same model on their own standard harness - a 37-point gap that is scaffolding, not model. OpenAI also edited published figures after release (hallucination rate 4.2% to 2% and back to 4.2%), and Stanford researchers raised 'benchmaxxing' concerns. Against that, Francois Chollet - who built the benchmark and has no stake in OpenAI - said progress came about twice as fast as he expected and moved his AGI forecast earlier. Genuine disagreement, not a settled result. || ⚠️ THE ANNOUNCEMENT SAYS NOTHING ABOUT CHIPS. Not one word about GPUs, silicon, data centres or Stargate. Every compute deal being quoted alongside this news predates Astra: NVDA 10GW (Sep 2025), AMD 6GW plus a 160m-share warrant (Oct 2025), the Broadcom-built Jalapeno chip (Jun 2026), AWS 38bn (Nov 2025), ORCL over 300bn (Sep 2025), Azure 250bn with a 27% stake (Oct 2025). 'Buy a chip stock because of Astra' is a narrative, not a fact - the contracts were signed long before. || ⚠️ AND THE MARKET-REACTION STORY IS CONFOUNDED. No sourced attribution of any share-price move to Astra was found. NVDA announced the acquisition of Hugging Face for 12.93bn on the SAME DAY. Any Sep 3-4 move cannot be cleanly assigned to Astra, and for NVDA the acquisition is plausibly the larger news. || WHERE THE REAL LINK IS: token consumption. Agents running 40-minute autonomous tasks burn far more tokens than chat, at 2.5x the price. That feeds inference silicon, memory, interconnect and power over 12-24 months - it does not show up in a two-day price move. Most direct listed beneficiaries in this book are MSFT (27% owner of OpenAI, Azure serves Astra), AMZN (Bedrock serves Astra, 38bn deal) and ORCL (largest contract, weakest balance sheet). || THE UNDER-OWNED ANGLE IS CYBERSECURITY, and it is the only causal chain Astra actually created rather than inherited. First model ever rated Critical for cyber capability. CRWD and PANW carry only 0.66% and 0.63% of the book with 12,325 of combined room. Rungs added to this Schedule, both conditional on results, not on the theme. || ON THE 'AI KILLS SAAS' STORY: not substantiated for Astra. The piece being circulated is dated Feb 10, 2026, seven months before Astra existed. Our own Aug 29 review found all eleven SaaS names raised or maintained guidance and none blamed AI. || NO POSITIONS, BUDGETS OR PRICES CHANGED. No trade is recommended on this news alone. || Sep 5, 2026 - BOARD FOCUSED AT SALEE'S INSTRUCTION. He asked to cut the watchlist back to names that fit a 5-10 year growth mandate and to free up attention. 46 further names removed, taking the board 178 -&gt; 132: 26 loss-making or shrinking small caps with no path to profit, the 5 remaining bitcoin miners as off-thesis, 14 mature low-growth names that cannot compound at the required rate, and Nu Holdings for consistency with the Sep 5 decision to take Brazil out of the allocation. Watchlist 126 -&gt; 80; 52 held positions untouched. || BUDGETS WITHDRAWN: Planet Labs 10,000 and McDonald's 5,000. Allocated budget therefore falls 1,000,000 -&gt; 985,000, leaving 15,000 to be re-assigned to names that meet the mandate. || SIX HOLDINGS MARKED FOR LIQUIDATION at Salee's instruction, recorded on the Schedule tab as SELL rows. Claude does not and will not place trades - Salee executes these at POEMS. Tesla (revenue +2.3%, EPS -37.4%, 163x forward), Intel (revenue +1.4%, loss-making, 86x forward, sold into a +112% gain), Ondas (going-concern doubt), Applied Optoelectronics (loss-making at 55x forward), IREN (bitcoin miner, -99.4% net margin) and Qualcomm (revenue +5.2%, EPS -6.3%). Combined proceeds ~14,161 at the Sep 4 close for a net gain of ~763 across the six. || ⚠️ THE STATED REASON WAS WRONG AND SALEE SHOULD KNOW IT. He asked to sell in order to free liquidity. He does not need liquidity: 402,694 of the 1,000,000 budget is still unspent and another 200,000 arrives on Sep 14. The valid reason to sell these six is quality and attention, not funding. Positions and costs are unchanged until he reports the fills. || Sep 5, 2026 - WATCHLIST CLEAN-UP BEGINS at Salee's instruction. He asked to cut the board back to names that fit a 5-10 year growth mandate, saying 129 watchlist names were too many to digest. Three removed on his explicit list: MELI (consistent with the Sep 5 decision to take Brazil out of the allocation entirely), SOUN (no path to profit - net margin -67.5%, return on equity -32.2%) and UBER (a sound business but revenue growth 16.7% with earnings per share falling 22.5%, and off-thesis for this book). Board 181 -&gt; 178 names, 52 held, 126 watchlist. No positions, budgets or prices touched. A tiered proposal for the remaining cut, plus liquidation candidates among the held names, has been put to Salee and awaits his decision. || Sep 5, 2026 - R&amp;D SPENDING RECORDED FOR THE SEVEN MEGA-CAPS at Salee's request, saved to the per-stock notes page. Latest reported fiscal year, US$ millions, every figure independently verified against SEC filings: AMZN 108,521 (+22.6%) - GOOGL 61,087 (+23.8%) - META 57,372 (+30.8%) - MSFT 35,562 (+9.5%) - AAPL 34,550 (+10.1%) - NVDA 18,497 (+43.2%) - TSLA 6,411 (+41.2%). The six genuine research lines total 213,479. || ⚠️ AMZN's 108,521 is its 'technology and infrastructure' line, not research and development. Amazon reports no R&amp;D line at all - the tag does not exist in its SEC XBRL data - and that bucket also carries the running costs of AWS infrastructure. Amazon leading this chart is an artifact of how the line is drawn, not research intensity, and it must not be set beside the other six. || ⚠️ THE SOURCE GRAPHIC WAS WRONG ON MSFT. It printed 32,488 (+10.1%), which is fiscal 2025 ended Jun 30 2025. Fiscal 2026 ended Jun 30 2026 and the 10-K was filed Jul 29 2026, before the graphic's own stated August 2026 cutoff, so the current figure was available and was not used. The true number is 35,562 (+9.5%), which also lifts MSFT above AAPL to 4th place. Six of the seven figures matched the filings to the dollar; only MSFT did not. || Fiscal calendars are not aligned - NVDA's year ended Jan 25 2026, MSFT's Jun 30 2026, AAPL's Sep 27 2025, and the rest Dec 31 2025 - so this is not a like-for-like comparison of the same twelve months. No board fields, budgets or positions were changed; this is reference information only. || Sep 6, 2026 - MU STRATEGY REVISED. Micron closed at 1,016.59 on Sep 4, through the 1,000 level, +244.5% year-to-date from a Jan 2 base of 295.13 and 19.0% below its 1,255 high. Salee's position - 35.45 shares at an average of 636.998 - is now worth ~36,038 for a gain of ~13,457, up 59.6%. Room unchanged at 7,418.42 on a 30,000 budget; 3.78% of the book. || ⚠️ A FLAW IN MY OWN PLAN, CORRECTED. The standing MU limit order at 750 now sits 26.2% BELOW the market. It would almost certainly never fill, and if it did, a 26% collapse would be a reason to RE-UNDERWRITE the position, not to buy automatically. A rule that cannot fire is not a rule. It has been DELETED and replaced with an evidence-based second rung: 3,418.42 at the Q1 FY2027 print (~mid-December), deployable ONLY if DRAM bit shipments grow double-digit for a SECOND consecutive quarter. Two in a row means the story has genuinely turned from price to volume; one is noise. The 30 Sep rung is unchanged at 4,000 on the same bit-growth test plus gross margin &gt;=80%. Total scheduled 7,418.42 = exactly the room. || ON THE 'SOLD OUT' HEADLINE, WHICH IS THE REASON THE STOCK IS RUNNING - it is weaker evidence than it looks. The claim that all 2027 DRAM and HBM capacity at Samsung, SK hynix and Micron is booked traces to DigiTimes citing 'industry insiders' (Aug 4, 2026), NOT to a Micron disclosure; the same report mentions long-term agreements of up to five years but states nothing about whether these are firm volume commitments, prepayments, or non-binding. Micron's own language in its prepared remarks is narrower: 'We expect tight conditions to persist beyond calendar 2027' - a statement about DURATION, not about being sold out. || ⚠️ THE DISTINCTION THAT MATTERS: being sold out is about ALLOCATION, not PRICE. Fully committed capacity does not stop contracts repricing lower at renewal, and TrendForce has DRAM contract price growth decelerating from +90-95% (1Q26) to +58-63% (2Q26) to +13-18% (3Q26). Micron's own CFO disclosed DRAM bits up 'low-single-digit percentage range' while prices rose in the 'low-60s' - roughly 95% of revenue growth is price. FY2023 remains the precedent: revenue halved from 30,758m to 15,540m and gross margin went NEGATIVE 9.1% on a 5.83bn loss. || CREDIT WHERE DUE - the source post was responsibly balanced, naming cyclicality, a possible supply glut, competition from SK hynix and Samsung, and valuation risk after the rally. Its '+200% from ~315' is an understatement: Jan 2 295.13 to the 1,255 high is +325.2%. || A TRIM IS NOW A LIVE OPTION, RECORDED NOT RECOMMENDED. Analyst fair value spans 361 to 2,200 across 45 analysts - a 6x spread, which IS the cycle uncertainty made visible. Taking something off the table before Sep 30 is a legitimate choice and Salee's to make. Added as a standing HOLD line on the Schedule tab so it is visible rather than forgotten. || Sep 5, 2026 - BOARD BROUGHT TO EXACTLY 1,000,000 at Salee's instruction to follow the standing budget recommendations. Two budgets withdrawn, 5,000 each, both ZERO deployed so no position is stranded and no money moves. Assigned budget 1,010,000 -&gt; 1,000,000, i.e. 100.00% of target for the first time since LHX and FPS were added. Unfilled room 412,694.31 -&gt; 402,694.31. || (1) ZS ZSCALER - budget 5,000 -&gt; None. Flagged as the standing trim candidate on four separate occasions and the reason is now explicit in the data: it is the ONLY LOSS-MAKING name of the three cybersecurity holdings, net margin -1.88% and ROE -2.43%, against PANW and CRWD which are both already deployed and both showing large gains (+94% and +120% respectively). Forward P/E 36.55 with a PEG of 1.39. Group 15 Cybersecurity 25,000 -&gt; 20,000, which is still 2x its deployed 7,675. CONSEQUENCE: ZS was a 5,000 line in TRANCHE 1 of the deployment plan, so Tranche 1 falls 75,697 -&gt; 70,697 and the whole plan 197,311 -&gt; 192,311. The buffer rises correspondingly. || (2) AMPX AMPRIUS TECHNOLOGIES - budget 5,000 -&gt; None. Net margin -43.98% and ROE -44.16% on a 9.89 share price; revenue growth of 172.6% is off a very small base. It was the fifth name in group 8 Defence, Drones &amp; Public Safety, behind PLTR (5,533 deployed), AVAV (3,758), ONDS (2,031) and LHX (5,000 budgeted at Salee's own instruction). Group 8 budget 30,000 -&gt; 25,000. Nothing was deployed and no thesis was ever written for it. || WHY THESE TWO AND NOT OTHERS - every other zero-deployed budget was protected for a stated reason: V and MCD are dated Tranche 1 lines; APP, PL, LUNR, FPS and LHX all carry explicit triggers set within the last three days; IONQ is the board's ONLY quantum name, so cutting it would delete a whole theme rather than trim a duplicate; CAT and AEP are profitable industrials (ROE 56.97% and 10.13%). ZS and AMPX were the only zero-deployed budgets that were BOTH loss-making AND redundant inside an already-funded group. || CONSIDERED AND REJECTED - ONDS was the other candidate on thesis grounds (previously recorded as carrying 'substantial doubt' language and +156% dilution), but it has 2,030.54 deployed, so trimming it would have been a partial cut rather than a clean withdrawal, and its board fields look internally suspect (pm 251.92%, roe 42.95% sit oddly against that thesis). Flagged for the fundamentals job to re-verify rather than acted on with data I do not trust. It remains the next candidate if the target is ever cut below 1,000,000. || Held positions 52 and held cost 597,305.69 UNCHANGED. AI concentration unchanged at the held level - this removes future headroom, not money. Board 181 tickers. || Sep 5, 2026 - THREE APPROVED BOARD ACTIONS EXECUTED TOGETHER at Salee's instruction. || (1) SPACE FUNDED BY TRIMMING TWO ON-HOLD AI-CORE NAMES. ALAB 15,000 -&gt; 7,000 (-8,000) and LITE 20,000 -&gt; 13,000 (-7,000); both budgets remain ABOVE their deployed cost (ALAB 3,805.47, LITE 9,372.74) so no position is stranded. The 15,000 goes to group 7 Space, which rises 10,000 -&gt; 25,000: RKLB unchanged at 10,000 (1,942.58 deployed), PL Planet Labs NEW 10,000, LUNR Intuitive Machines NEW 5,000. RATIONALE - ALAB (fwd P/E 86.95) and LITE (ROE -149.3%) have both been on explicit hold for weeks, so their budgets were dead money; Space carried 1.00% of a 1,005,000 target across six names, too little to express any view. This single move funds the theme AND reduces AI-core budget, addressing the standing concentration problem from both ends. PL is the only name in the group approaching profitability - Q2 FY27 revenue 116.1m +58%, adjusted EBITDA POSITIVE 13.9m, GAAP loss narrowed from -22.6m to -9.4m, cash 865.4m against 448.3m of converts, backlog 814.9m. CAVEAT: PL guided next quarter to 101-105m against 114.3m consensus, a sequential DECLINE - hence the trigger is the ~December print, not now. LUNR revenue tripled to 206.2m with an 1.8bn backlog but debt went 37m -&gt; 481m and shares +44.1% YoY; trigger is IM-3 actually flying. SPCX and ASTS deliberately left unfunded (82x sales; a 231m quarterly loss with debt +492%). || (2) APP BUDGET SET AT 5,000. This corrects a documented discrepancy: the 200k deployment plan has stated since Sep 3 that APP had a 5,000 budget, but the board carried None - the intent was written and never executed. Recorded as an error, not a change of view. NOTHING DEPLOYED - the trigger remains the ~Nov 4 print. WHY APP IS CHEAP, NOW ESTABLISHED: the fall from 745.61 to ~320 is DECELERATION, not fraud. Revenue growth ran 68% -&gt; 66% -&gt; 59% -&gt; 53% -&gt; guided 47%, culminating in a -19.66% day on Aug 6 2026 after the first-ever guidance miss (Q2 revenue 1,924m vs ~1,935m consensus). CEO Foroughi: 'Our pace of meaningful model improvement was lighter than normal during the quarter, and the next step up in model performance landed just after quarter end.' TWO OVERHANGS HAVE RESOLVED IN APP'S FAVOUR - CFO Matt Stumpf stated Aug 5 2026 that 'The SEC has recently advised us that it concluded its inquiry with no recommended action', and CapitalWatch RETRACTED its money-laundering report on Feb 9 2026 citing a 'flawed verification process'. The 2025 Fuzzy Panda/Culper class action remains at motion-to-dismiss, undecided. Short interest only 3.9% of float. Business quality intact: Q2 gross margin 88.3%, net income 1,267m +55%, free cash flow 863m in the quarter. || (3) SIDU REMOVED FROM THE BOARD. Sidus Space had no budget and no position, so nothing is lost. Q2 2026 revenue FELL 54% to 583k while every peer in the group grew; gross margin is NEGATIVE 108%; share count went roughly 18.30m -&gt; 101.21m in twelve months; the company executed a 1-for-100 reverse split in Dec 2023 to regain Nasdaq minimum-bid compliance. It was a row producing noise, not signal. Board 182 -&gt; 181 tickers. || ⚠️ FOUR APP FIELDS ARE WRONG ON THIS BOARD and are flagged for the next fundamentals pass, NOT silently patched here: fpe carried as 24.17 but the true FORWARD P/E is 17.72 (24.65 is the TRAILING multiple); roe carried as 266.44 vs 203.69 sourced; de carried as 1.63 vs 1.11 (3.52bn debt / 3.16bn equity at Jun 30 2026); revG carried as 66.4 which was the Q4 2025 rate - the Q2 2026 YoY is 53%. Recorded rather than corrected because fundamentals belong to the earnings-refresh job. || ⚠️ BUDGET CONSEQUENCE - assigned budget 1,005,000 -&gt; 1,010,000, i.e. 101.0% of the 1,000,000 target. The Space reallocation was budget-NEUTRAL by construction (-15,000 AI core, +15,000 Space); the whole +5,000 is the APP line. ZS remains the standing trim candidate (5,000 budgeted, 0 deployed, weakest of the three cybersecurity names) which would return the board to 1,005,000; a further 5,000 trim is still needed for exactly 1,000,000. Salee has not yet chosen either, so the overage stands and is flagged, not absorbed. || Held positions 52 and held cost 597,305.69 both UNCHANGED - these are budget and roster changes, no money moved. Unfilled room 412,694.31. || Sep 4, 2026 - close. Daily price refresh: 160 of 182 tickers brought to the Friday Sep 4, 2026 close (price, mcapB, pxd; mcapB scaled by each ticker's exact price ratio). METHOD per playbook: stockanalysis.com quote page taken only when stamped "Sep 4, 2026, 4:00 PM EDT" AND its stated previous close tied to the Sep 3 close; partial-session /history/ rows discarded throughout (worst: SITM history close 611.07 above its own high 608.58 - internally impossible; MCD history close below its own low; KTOS/ONDS/RCAT/RBRK/SOUN/WULF/PENG/YUM/BKNG/S rows were low-volume partial captures, quote page used); history-table fallbacks for MMM and FSLR (quote pages intraday-stamped, Sep 4 rows internally consistent); GOOGL prev-close tie via the Sep 3 adjusted close (0.22 dividend adjustment). CONSTRAINT THIS RUN, RECORDED RATHER THAN PAPERED OVER: the session's 200-call WebSearch budget was exhausted mid-run by the 182-ticker fan-out, which also blocks provenance for new second-source URLs, so most late-batch names could not reach Google Finance/marketscreener/ycharts/fool. All 23 moves &gt;=6% were treated per the gate. ELEVEN confirmed against dated independent Sep 4 sources and passed with --allow: AEHR +13.1% (marketscreener), EOSE +10.9% (Google Finance beta 'Closed: Sep 4, 4:00:01 PM GMT-4'), ALAB +9.8%, AXTI +9.7%, POET +8.1%, TSEM +7.9%, NBIS +7.5%, FORM +7.4%, MRVL +7.1%, COHR +6.6% (all Google Finance dated closes), MU +6.1% (GF beta, prev close derived per the after-hours quirk). TWELVE &gt;=6% moves could NOT be second-sourced and were REVERTED to their Sep 3 board values per the stale-beats-wrong rule - each had an internally consistent single-source Sep 4 print (4:00 PM EDT stamp + prev-close tie, most with an exactly agreeing history row) that the next run should confirm and apply: SNDK 1740.00 (+11.9%), COHU 50.72 (+10.3%), SKHY 177.00 (+8.1%), KLAC 185.60 (+7.3%), IREN 44.68 (+7.3%), BE 252.87 (+7.3%), SITM 612.09 (+6.5%), PENG 51.76 (+6.4%), NRG 119.02 (+6.4%), ADBE 266.51 (-6.7%; two Sep-4-dated headlines corroborate a ~7% fall on CEO-succession disappointment but no fetchable second quote), STX 849.28 (+6.3%), HUT 93.55 (+6.2%). Their pxd stays 2026-09-03 so the staleness badges show honestly. UNRESOLVED, left at prior values: POWI/AMBQ/INDI/KEEL/OSS - quote pages pinned to intraday snapshots across repeated cache-busted fetches, no valid Sep 4 history rows; CLPT - no Sep 4 print anywhere reachable (Sep 3 after-hours was +4.6%, so the stale value was deliberately not nudged); FPS/HYLN/AIRJ - stockanalysis never posted their Sep 4 session; VPG - quote page cleanly stamped Sep 4 (63.01) but its previous-close linkage (implied Sep 3 close 62.76) unverifiable against any source - same precedent as HNGE on Sep 3, not used. VIAV UNSTUCK at 34.86 (marketscreener 'Market Closed 2026-09-04' concurs exactly). HNGE UNSTUCK at 92.37 (linkage rebuilt: Sep 1 90.02 confirmed, quote prev close 90.76 for Sep 3; a fool.com quote box concurs on price and the 89.41-93.14 day range, though its date label read Sep 3 and its derived prev close 90.60 differs 0.18% - accepted on the strength of the at-close stamp + range agreement, caveat recorded). Movers 5.5-6% (under gate, single-source, recorded): TSLA -5.9%, WDC +5.9%, STRL +5.8%. hi52/lo52 extended from sourced Sep 4 session extremes where breached. NOTE: first push attempt was rejected - another writer (the Sep 5 Brazil-removal commit) landed first; this build was redone on top of it per the README recovery protocol. Fundamentals, M3, POS, TRADES, budgets untouched (owned by other jobs). Also recorded: this session's git proxy would not inject a credential for this repo ('not in this session's authorized repository set'); the push used the job's own PAT explicitly. || Sep 5, 2026 - BRAZIL REMOVED FROM THE ALLOCATION at Salee's explicit instruction. NU (Nu Holdings) keeps its board row and all research, but its 5,000 budget is withdrawn, so it cannot be bought. Group 14 Digital Fintech goes 10,000 -&gt; 5,000 (V only). Total assigned budget 1,010,000 -&gt; 1,005,000. Tranche 1 of the deployment plan falls 80,697 -&gt; 75,697; the whole plan 202,311 -&gt; 197,311; buffer ~11,747 -&gt; ~16,747. || THE FACTS DO NOT SUPPORT THE STATED REASON, AND THIS IS RECORDED HONESTLY. Salee cited Brazilian economy, inflation and currency. All three currently point the other way: IPCA 4.44% (Jul 2026) sits INSIDE the 3.0% +/-1.5pp tolerance band, and the Aug IPCA-15 preview showed outright monthly DEFLATION of -0.40% with the 12-month rate easing to 4.24%; the Selic is being CUT not raised - four consecutive 25bp cuts in 2026 taking it 15.00% -&gt; 14.00%, the last unanimous 7-0 on Aug 5; GDP grew +0.5% QoQ and +2.0% YoY in Q2 2026, above expectations; and the real APPRECIATED against the dollar, +6.1% over 12 months on BCB PTAX and +3.4% on the Fed's H.10, leaving it 1.4% STRONGER than five years ago. On identical Fed H.10 dates the Brazilian real (+3.4%) outperformed BOTH the Taiwan dollar (-3.5%) and the Thai baht (-3.4%) - Salee's own currency weakened more than the one he is avoiding. || TWO REAL CONCERNS EXIST, NEITHER ON HIS LIST - (1) general government gross debt has climbed without interruption from 75.49% of GDP in Jan 2025 to 82.51% in Jul 2026, nearly 4pp of that in 2026 alone; (2) Brazil is BELOW investment grade at all three agencies (Fitch BB, Moody's Ba1, S&amp;P BB/B, all Stable), and a general election falls on Oct 4 2026 with a runoff Oct 25 - Nu's own FY2025 20-F names that election as a risk factor. || NUBANK ITSELF - Brazil is 117.8m of 138.9m customers (84.8%) and 36.4bn of 45.3bn deposits (80.4%); revenue by geography is NOT disclosed. Two disclosed offsets cut against the currency fear: Nu's functional AND presentation currency is the US DOLLAR, and real appreciation FLATTERED its reported results (revenue +55.8% in USD vs +39% FX-neutral); and its cost of deposits runs at 88% of the Brazilian interbank rate, so a FALLING Selic mechanically lowers funding cost. The one genuinely deteriorating metric is 90+ NPL at 6.9%, up 35bp QoQ and 40bp YoY, while the leading 15-90 day indicator IMPROVED 16bp to 4.8%. || WHY THE DECISION STILL STANDS - not because Brazil is unstable, but because 5,000 is 0.5% of a 1,000,000 target. Tripling it would add 1% to the portfolio, which cannot justify holding something Salee has no information flow on and cannot monitor. A position too small to matter and too uncomfortable to hold is sold at the wrong moment. Recorded so that the reasoning is not later mistaken for a macro call on Brazil. || MELI (MercadoLibre) is the only other LatAm row on the board and already carries NO budget, so it is already outside the allocation; Salee sold his position earlier. No further action taken. Held positions 52 and held cost 597,305.69 both UNCHANGED - this removes budget, not money. || Sep 3, 2026 - close. Daily price refresh: 180 of 182 tickers brought to the Thursday Sep 3, 2026 close (price, mcapB, pxd; mcapB scaled by each ticker's exact price ratio; FPS and VPG only to their verified Sep 2 close - their Sep 3 pages never posted). METHOD per playbook: stockanalysis.com quote page taken only when stamped "Sep 3, 2026, 4:00 PM EDT" AND its stated previous close tied to the Sep 2 close; partial-session /history/ rows discarded throughout (MCHP history close 72.74 above its own high 72.65 - internally impossible; CGNX history close 58.90 below its own low 59.21 - impossible; YUM/MMM/ROK/SOUN/IBM/FN/PENG/OKTA/S/CCJ/UUUU/NU/CRCL history rows were low-volume partial captures, quote page used). Intraday-stamped quote pages for ON (3:09 PM), SITM (2:13 PM), MTSI (12:19 PM), YUM (12:41 PM) resolved via the history table or dated Google Finance closes; stale stockanalysis caches for POWI/AMBQ/COHU/CLFD/AXTI/POET/QNT/TSEM/FORM/OSS/CLPT/LMND/AIRJ resolved via dated Google Finance / marketscreener closes with previous-close linkage proving the day. ALL 31 moves &gt;=6% vs the previous build second-sourced against dated Google Finance closes (or marketscreener/ycharts where GF caches were stale): DELL +21.5% and HOOD +20.5% (post-earnings/upgrades), CIFR +18.9%, RIOT +18.8%, EOSE +15.1%, CRCL +15.4%, HUT +13.6%, IREN +13.1%, SNOW +11.5%, ASTS +11.3%, CORZ +11.4%, WULF +10.8%, BE +10.3%, KEEL +9.1%, ORCL +9.0%, SYM +8.8%, SOFI +8.6%, NU +8.4%, PYPL +8.4%, ONDS +8.4%, OUST +7.7%, LMND +7.3%, HYLN +7.0%, HPE +7.0%, APLD +6.7%, AFRM +6.2%, TE +6.1%, AMBA -6.6%, PANW -8.3%, MDB -11.5%, CIEN -11.9% (post-earnings selloff despite record Q3). APH: the 2-for-1 split was applied by the Sep 4 POEMS reconciliation job; this refresh prices it at the split-adjusted Sep 3 close 82.07 (stockanalysis quote validated, Google Finance 'Closed: Sep 3, 4:00:09 PM GMT-4' concurs; +0.59% vs the split-adjusted Sep 1 base 81.59). UNRESOLVED, left at prior values: VIAV - quote page frozen intraday (2:27 PM), history stale, both Google Finance caches stale; no dated Sep 3 close found. HNGE - quote page stamped Sep 3 but its previous close could not be validated against any source (history and GF end Aug 31); unvalidated 90.76 NOT used. hi52/lo52 extended from sourced Sep 3 session extremes where breached. Fundamentals, M3, POS, TRADES untouched (owned by other jobs). || Sep 4, 2026 - POEMS reconciliation. Two changes, both verified against the broker screenshot to the last decimal. || (1) AVGO POSITION ADDED TO. Limit BUY 343.50 filled at 343.352 for 4.5 shares, order O9636090382424019, submitted and completed Sep 3 2026 10:53:44 PM SGT. Lot cost 1,553.65 = 4.5 x 343.352 (1,545.09) + the flat 8.56 POEMS commission. Position 84 -&gt; 88.5 shares, cost 28,571.53 -&gt; 30,125.18, average 340.14 -&gt; 340.39751 - ties exactly to the POEMS average price field. Budget room 40,000 - 30,125.18 = 9,874.82 (was 11,428.47). Broadcom sits in group 1 and this was Salee's own trade, taken after AVGO's Sep 2 AMC print in which AI semiconductor revenue was 16.7bn, +221% YoY, with Q4 guided to 21.7bn. || (2) APH TWO-FOR-ONE STOCK SPLIT - CAUGHT BY RECONCILIATION, NOT PREVIOUSLY ON THE BOARD. POEMS shows 32 shares against the board's 16 at an IDENTICAL cost of 2,004.40, which is the signature of a split rather than a purchase. Confirmed against Amphenol's own investor-relations release dated Aug 6 2026: </t>
+          <t>Sep 7, 2026 - WEEKLY REFRESH &amp; INTEGRITY AUDIT. Prices verified at the Fri Sep 4 close (US markets closed Mon Sep 7, Labor Day). PENG applied at 51.76 (+6.44%), the one name the Sep 4 daily job left unconfirmed - second-sourced via stockanalysis.com and Google Finance, mcapB scaled to 2.6528 by the same ratio. QNT hi52/lo52 filled (86.79/46.54, stockanalysis.com) - they were null on a listed stock. SPCX and QNT listings independently re-verified (SpaceX IPO Jun 12 2026 Nasdaq, Quantinuum IPO Jun 2026 Nasdaq; prices/mcaps match the board): the Sep 6 correction stands, the QNT removal patch stays unapplied. AUDIT: implied share counts clean (only APH moved, 2-for-1 split Sep 4, expected); no ticker flat 7+ days; NASD 493,545.18 + NYSE 103,760.51 = 597,305.69 ties exactly; REALIZED/SOLD/MONTHLY byGroup mutually consistent (known NBIS 1-cent and sale-time-group semantics unchanged). FLAGGED, NOT FIXED: (1) four Aug 5-7 fills (TSM 4.5sh, NVDA 9sh, CRM 10sh, ISRG 5sh) imply ZERO commission - amount equals shares x price exactly, and the per-share prices look back-computed from the amount; every other fill since Jul 28 implies the flat 8.56. Either those four amounts omit the 8.56 (book cost understated ~34.24 total) or the price field folds commission in - needs the POEMS contract notes to settle; TRADES untouched, only Salee changes fills. (2) TOTALS identity drift: investedEver - soldCost - heldCost = -9,210.82, was -5,653.61 at the Aug 31 weekly; the -3,557.21 widening this week is roughly the Sep 4 AVGO +4.5sh reconciliation - investedEverUSD semantics vs booked cost should be pinned. (3) ath&lt;hi52 on 29 names - consistent with ath=highest CLOSE vs hi52=intraday, but the convention is still not pinned in the README. pe deliberately null on CRWD/FPS (near-zero eps). || Sep 6, 2026 - MSFT RUNG ADDED, closing a genuine gap in the plan. Salee asked whether the four largest companies in a viral graphic had any place in the next three months of the schedule. Checking it exposed an oversight of mine: GOOGL had a dated tranche (20,524.08 on Nov 19, unlocked by the Oct 2 ad-tech judgment), NVDA had a rung plus two standing limits (8,000 on Nov 18, then 7,000 at or below 200 and 5,619.72 at or below 180), AAPL was deliberately parked on price - but MSFT, the third-largest holding at 52,878.96 with 7,121.04 of room, had NO row of any kind. It simply fell through when the tranches were built. A rung now sits on the Q1 FY2027 print. || ⚠️ THE DATE IS ESTIMATED, NOT CONFIRMED. Microsoft's investor site says only that the next release 'will be announced soon'. Oct 28 is inferred from the pattern - the last four reports were all Wednesdays (Oct 29 2025, Jan 28, Apr 29 and Jul 29 2026) - and one source says Oct 29 instead. Confirm before acting. || THE CONDITION IS NOT AZURE. Azure is guided to ACCELERATE to about 45% constant currency from 43%, and passed 100bn of annual revenue for the first time; Microsoft 365 Copilot passed 30 million paid seats. That part works. The risk is the spend: capex was 115.9bn in FY2026 against guidance of approximately 175bn for FY2027, up about 51%, while total revenue is guided at 16-17%. Deploy only if Azure holds the guided ~45% AND the 175bn capex number is not raised again. || ⚠️ AND THE GRAPHIC SALEE SENT WAS WRONG ON SEVEN OF EIGHT FIGURES. Verified against two independent sources: it showed MSFT at 2.92T against a true 3.71T (-21%), AAPL 4.05T against 4.67T (-13%), GOOGL 3.77T against 4.14T (-9%) and NVDA 4.44T against 5.56T (-20%). Its 2015 bases were wrong too - MSFT was 443B not 391B, AAPL 587B not 531B. Worse, none of its four multipliers reconciles with the two numbers printed directly above it: 2920 divided by 391 is 7.47, not the 6.69 shown. The true multipliers are MSFT 8.4x, AAPL 8.0x, GOOGL 7.7x and NVDA 313.6x - the bad arithmetic had ranked AAPL the weakest compounder when it actually beat GOOGL. The board's own market caps matched the verified figures on all four. || Sep 6, 2026 - ⚠️ CLAUDE WAS WRONG ABOUT SPCX AND HAS CORRECTED IT. On Sep 5 I told Salee that SPCX was probably a bad board entry because 'SpaceX is a private company', and I called the 2,007.68 market cap absurd. BOTH STATEMENTS WERE FALSE AND THE BOARD WAS RIGHT. SpaceX completed its IPO on Jun 12 2026 at 135 dollars a share, trades on Nasdaq under SPCX, and SEC EDGAR confirms CIK 0001181412 with ticker SPCX and exchange Nasdaq. Market cap at the Sep 4 close was 2.01 trillion - the board's figure was accurate to three decimal places. My knowledge cutoff is May 2026 and the IPO happened in June; I asserted a post-cutoff fact from memory instead of checking it, which is precisely the error I keep flagging in other people's graphics. || ⚠️ CONSEQUENCE FOR QNT: the same Sep 5 flag claimed Quantinuum was private too. That reasoning is now untrustworthy. A cloud session prepared a QNT removal patch on Sep 6 which has NOT been pushed. DO NOT APPLY IT until QNT's listing status is independently verified. QNT stays on the board for now. || ON THE VIRAL GRAPHIC Salee sent ('SpaceX stock eyes 48% rally as Starship Flight 14 and 280 target fuel bullish outlook'): the ticker is real and every number traces to a real source, but they are spliced into a claim no analyst makes. The 48% is upside to the CONSENSUS AVERAGE target of 222.32 across 35 analysts. The 280 is Oppenheimer alone (Tim Horan, Sep 2-3, raised from 250), which implies about 87-89% from the 147.95 close - not 48%. Putting the two side by side welds a consensus percentage onto an outlier bank's target. The 'BUY' badge is the consensus rating; Oppenheimer's own rating is reported as Outperform or Overweight, not Buy. || ⚠️ AND FLIGHT 14 HAS NOT FLOWN. It is no-earlier-than Sep 15 2026 per an FCC filing dated Aug 31. The graphic presents an unflown, un-de-risked test as an accomplished catalyst. The most recent flight is Flight 13 on Jul 24: the ship deployed 20 Starlink V3 satellites and survived splashdown intact for the first time, but the booster relit only 10 of its engines and was destroyed on water impact. That is a partial success, not a clean one. || WHAT THE GRAPHIC OMITS: SPCX at 147.95 trades BELOW its 161 first-day close. Q2 showed a 541m net loss on 15.83bn of AI capex against 2.56bn of AI revenue. Net margin is -35.66%. Analyst targets span 117 to 450 with one house at 800. || NO POSITION, BUDGET OR PRICE CHANGED. No budget assigned to SPCX. Two Schedule rows added: Flight 14 as a WATCH that explicitly is NOT a buy trigger, and a standing row saying wait for a second public quarter before assigning any budget. || Sep 6, 2026 - RKLB BUY PLAN RESTRUCTURED ON THE SCHEDULE TAB at Salee's instruction, replacing the single Tranche-2 line (8,057.42 dated Oct 9) with three rungs totalling exactly the room: (1) LIMIT 2,000 at any close &lt;=55; (2) TRIGGER 2,000 on the Iridium financing pricing day, deployable only if total equity dilution &lt;=15% - the $8.0bn deal's $3.6bn bridge loan is the live overhang (S-4 filed Aug 13, 'capital strategy underway'); (3) TRIGGER 4,057.42 after de-risking - a successful Neutron first flight (the 'Q4 2026' date is pad delivery, not launch) or deal close on sane terms. Rationale recorded: Berenberg's Sep 3 initiation (Buy, PT 83, 'most compelling and differentiated long-term asset in the space sector') is a real note but sits BELOW the 18-analyst mean of 112.94 - a conservative Buy, and no reason to chase a +12% day. Position 23 sh at 84.46 avg (-24%); the plan forbids averaging down beyond rung 1 merely to repair the lot. The Nov 9 RKLB earnings WATCH row is unchanged. No prices, budgets, positions or other tabs touched. || Sep 6, 2026 - WEEKLY REFRESH AND INTEGRITY AUDIT. The Sep 4 daily job reverted twelve &gt;=6% movers it could not second-source before its search budget ran out; this weekly run re-verified them. TEN CONFIRMED against a second independent dated source and applied at the Friday Sep 4 close with --allow, mcapB/pe/fpe/ps/peg rescaled by the exact price ratio per convention: SNDK 1,740.00 +11.90% (Google Finance 'Closed Sep 4, 4:00 PM GMT-4' agrees with stockanalysis to the cent), SKHY 177.00 +8.14% (GF + stockanalysis agree; the 24/7 Wall St intraday 174.38 was pre-close), BE 252.87 +7.35% (Motley Fool article of Sep 5 quotes 252.87 +17.32 exactly), KLAC 185.60 +7.32% (GF concurs, prev close ties to 172.94), IREN 44.68 +7.27% (GF dated close, +3.03 ties to the 41.65 board value), ADBE 266.51 -6.73% (24/7 Wall St Sep 4 CEO-succession piece quotes 266.51 -6.73% verbatim; GuruFocus concurs on a ~6-7% Friday fall), FPS 31.35 +6.56% off the Sep 2 close (Motley Fool at-close quote; GF intraday 31.44 at 11:29 AM concurs on level - accepted on the HNGE precedent, caveat recorded), SITM 612.09 +6.55% (Fool quote page shows 612.09 dated Sep 4 exactly, CAVEAT: its own day-change figure +1.07% implies a different Sep 3 close than the board's 574.47 - price corroborated, prior-day linkage not), NRG 119.02 +6.42% (GF dated close + Fool concur, open 111.29 ties to the board's 111.84 Sep 3 value), STX 849.28 +6.34% (GF dated close +50.67 ties exactly). ONE NOT CONFIRMED: PENG - GF still shows the Sep 3 close 48.63, Yahoo is stuck at Sep 1, CNN unusable; the pending 51.76 single-source print stays UNAPPLIED per the stale-beats-wrong rule and PENG remains at 48.63 with pxd 2026-09-03 showing honestly. Next daily run should confirm it. || AUDIT RESULTS, the checks the daily jobs cannot do. CLEAN: implied share counts (mcapB/price) moved &lt;1% on every name against the Aug 31 weekly build except APH, which doubled - the known 2-for-1 split applied in the Sep 4 POEMS reconciliation, correct; no ticker's price is stuck 7+ days (worst is PENG at 2 sessions); broker subtotals tie the Sep 4 POEMS screen to the cent - NASDAQ held cost 493,545.18 + NYSE 103,760.51 = 597,305.69; every fill since Jul 28 implies exactly the flat 8.56 POEMS commission (SKHY 8.57 / META 8.54 are fractional-share rounding); REALIZED, SOLD and MONTHLY byGroup are mutually consistent - July's byGroup ties byStock exactly under sale-time groups. FLAGGED, NOT FIXED: (1) NBIS realized gain is 1,404.52 in REALIZED but 1,404.51 in SOLD and MONTHLY - one cent, TOTALS ties to REALIZED; needs the POEMS figure to settle which. (2) Realized P&amp;L attributes to SALE-TIME groups: IREN g13, ORCL g10, SNPS g10, APP g10 predate the Aug 31 reclassification sweep (now g21/g13/g1/g19), so per-group realized figures reflect history, not today's grouping - semantics to be aware of, not corruption. (3) SNDK carries ath 1,804.00 BELOW hi52 2,354.39 and SITM ath 901.48 fractionally below hi52 901.81 - an all-time high cannot sit under a 52-week high unless ath means highest CLOSE and hi52 intraday; convention should be pinned and the two values re-sourced. (4) SNDK lo52 40.10 against a 1,740 price is a 43x 52-week range - plausible for the Feb-2025 spin-off in a memory supercycle but worth one look at POEMS. FIXED THIS RUN: the vestigial STOCKS.budget field had drifted from the authoritative POS budgets on 10 names (NVDA still showed 85,000 vs the 100,000 set Aug 27; FSLR, ONDS, IONQ, V, HUBB, AEP, SE, CAT, IREN showed None vs their 5,000 POS budgets) - synced to POS, which is what every page component actually reads, so nothing rendered changes. POS, TRADES, CASH, fundamentals untouched. IREN NOTE FOR THE SELLING TAB: the confirmed 44.68 close is 7.3% ABOVE the 41.65 carried on the IREN sell row; estimated proceeds there are now understated - no action taken, Salee executes. || Sep 5, 2026 - SELLING TAB ADDED at Salee's request as a control sheet for the liquidation programme. It carries, per name: shares, average cost, last close, target price or 'at market', estimated net proceeds, profit or loss, conviction, timing, the full reasoning, what happens to the budget after the sale, and a status of planned / placed / filled / cancelled. Estimated proceeds are net of the 8.56 flat POEMS commission - six sales cost 51.36 in total, which is why net proceeds are 14,110.13 against 14,161.49 gross, and net profit across the six is 711.69 rather than 763.05. || The sheet reads shares and cost live from the position book, so it cannot drift from the board, and falls back to stored values once a position is sold. A SELL DISCIPLINE panel records five standing rules, the first being: sell the thesis, not the price - three of the six are at a loss and one is up 112%, and that spread is deliberate. || ⚠️ THE TAB STATES PROMINENTLY THAT CLAUDE DOES NOT PLACE TRADES. Every row is an instruction for Salee to execute at POEMS; no position, cost or cash figure moves until he reports a fill. || Rows: TSLA and INTC at market (High conviction), ONDS at market with a limit if the spread is wide because the stock is thin (High), then IREN at 41.65, AAOI at 105.53 and QCOM at 168.74, all Medium and none urgent. || Build note: SELLBOOK was added to the CONSTS list in BOTH gen_dashboard.py and extract_data.py. A data block missing from either list is silently wiped on the next refresh. Verified by round-trip plus a headless Chromium render - no page errors, no horizontal overflow, all six reasoning blocks wrap without clipping. || Sep 5, 2026 - GPT-6 ASTRA ASSESSED (OpenAI, announced Sep 3). Salee asked whether it opens a new chapter for AI and who benefits. Five watch/decide rows added to this Schedule. || WHAT IT IS: a frontier model, not a new product category - 1,050,000 token context, 10 dollars in / 50 dollars out per million tokens (a 2.5x price rise), served on OpenAI's API, Azure and AWS Bedrock. The real advance is computer use: 72.6% on OSWorld in about 40 minutes per task versus 65.7% in about 75 minutes for the prior model. || ⚠️ THE 'STEP CHANGE' CLAIM IS CONTESTED AND SHOULD NOT BE TRADED AS FACT. Epoch AI ranked Astra first across 50+ tests; Artificial Analysis scored it flat versus its predecessor and BEHIND Anthropic's Claude Fable 5.1. OpenAI's headline 99.9% on ARC-AGI-3 was 62.7% when ARC Prize ran the same model on their own standard harness - a 37-point gap that is scaffolding, not model. OpenAI also edited published figures after release (hallucination rate 4.2% to 2% and back to 4.2%), and Stanford researchers raised 'benchmaxxing' concerns. Against that, Francois Chollet - who built the benchmark and has no stake in OpenAI - said progress came about twice as fast as he expected and moved his AGI forecast earlier. Genuine disagreement, not a settled result. || ⚠️ THE ANNOUNCEMENT SAYS NOTHING ABOUT CHIPS. Not one word about GPUs, silicon, data centres or Stargate. Every compute deal being quoted alongside this news predates Astra: NVDA 10GW (Sep 2025), AMD 6GW plus a 160m-share warrant (Oct 2025), the Broadcom-built Jalapeno chip (Jun 2026), AWS 38bn (Nov 2025), ORCL over 300bn (Sep 2025), Azure 250bn with a 27% stake (Oct 2025). 'Buy a chip stock because of Astra' is a narrative, not a fact - the contracts were signed long before. || ⚠️ AND THE MARKET-REACTION STORY IS CONFOUNDED. No sourced attribution of any share-price move to Astra was found. NVDA announced the acquisition of Hugging Face for 12.93bn on the SAME DAY. Any Sep 3-4 move cannot be cleanly assigned to Astra, and for NVDA the acquisition is plausibly the larger news. || WHERE THE REAL LINK IS: token consumption. Agents running 40-minute autonomous tasks burn far more tokens than chat, at 2.5x the price. That feeds inference silicon, memory, interconnect and power over 12-24 months - it does not show up in a two-day price move. Most direct listed beneficiaries in this book are MSFT (27% owner of OpenAI, Azure serves Astra), AMZN (Bedrock serves Astra, 38bn deal) and ORCL (largest contract, weakest balance sheet). || THE UNDER-OWNED ANGLE IS CYBERSECURITY, and it is the only causal chain Astra actually created rather than inherited. First model ever rated Critical for cyber capability. CRWD and PANW carry only 0.66% and 0.63% of the book with 12,325 of combined room. Rungs added to this Schedule, both conditional on results, not on the theme. || ON THE 'AI KILLS SAAS' STORY: not substantiated for Astra. The piece being circulated is dated Feb 10, 2026, seven months before Astra existed. Our own Aug 29 review found all eleven SaaS names raised or maintained guidance and none blamed AI. || NO POSITIONS, BUDGETS OR PRICES CHANGED. No trade is recommended on this news alone. || Sep 5, 2026 - BOARD FOCUSED AT SALEE'S INSTRUCTION. He asked to cut the watchlist back to names that fit a 5-10 year growth mandate and to free up attention. 46 further names removed, taking the board 178 -&gt; 132: 26 loss-making or shrinking small caps with no path to profit, the 5 remaining bitcoin miners as off-thesis, 14 mature low-growth names that cannot compound at the required rate, and Nu Holdings for consistency with the Sep 5 decision to take Brazil out of the allocation. Watchlist 126 -&gt; 80; 52 held positions untouched. || BUDGETS WITHDRAWN: Planet Labs 10,000 and McDonald's 5,000. Allocated budget therefore falls 1,000,000 -&gt; 985,000, leaving 15,000 to be re-assigned to names that meet the mandate. || SIX HOLDINGS MARKED FOR LIQUIDATION at Salee's instruction, recorded on the Schedule tab as SELL rows. Claude does not and will not place trades - Salee executes these at POEMS. Tesla (revenue +2.3%, EPS -37.4%, 163x forward), Intel (revenue +1.4%, loss-making, 86x forward, sold into a +112% gain), Ondas (going-concern doubt), Applied Optoelectronics (loss-making at 55x forward), IREN (bitcoin miner, -99.4% net margin) and Qualcomm (revenue +5.2%, EPS -6.3%). Combined proceeds ~14,161 at the Sep 4 close for a net gain of ~763 across the six. || ⚠️ THE STATED REASON WAS WRONG AND SALEE SHOULD KNOW IT. He asked to sell in order to free liquidity. He does not need liquidity: 402,694 of the 1,000,000 budget is still unspent and another 200,000 arrives on Sep 14. The valid reason to sell these six is quality and attention, not funding. Positions and costs are unchanged until he reports the fills. || Sep 5, 2026 - WATCHLIST CLEAN-UP BEGINS at Salee's instruction. He asked to cut the board back to names that fit a 5-10 year growth mandate, saying 129 watchlist names were too many to digest. Three removed on his explicit list: MELI (consistent with the Sep 5 decision to take Brazil out of the allocation entirely), SOUN (no path to profit - net margin -67.5%, return on equity -32.2%) and UBER (a sound business but revenue growth 16.7% with earnings per share falling 22.5%, and off-thesis for this book). Board 181 -&gt; 178 names, 52 held, 126 watchlist. No positions, budgets or prices touched. A tiered proposal for the remaining cut, plus liquidation candidates among the held names, has been put to Salee and awaits his decision. || Sep 5, 2026 - R&amp;D SPENDING RECORDED FOR THE SEVEN MEGA-CAPS at Salee's request, saved to the per-stock notes page. Latest reported fiscal year, US$ millions, every figure independently verified against SEC filings: AMZN 108,521 (+22.6%) - GOOGL 61,087 (+23.8%) - META 57,372 (+30.8%) - MSFT 35,562 (+9.5%) - AAPL 34,550 (+10.1%) - NVDA 18,497 (+43.2%) - TSLA 6,411 (+41.2%). The six genuine research lines total 213,479. || ⚠️ AMZN's 108,521 is its 'technology and infrastructure' line, not research and development. Amazon reports no R&amp;D line at all - the tag does not exist in its SEC XBRL data - and that bucket also carries the running costs of AWS infrastructure. Amazon leading this chart is an artifact of how the line is drawn, not research intensity, and it must not be set beside the other six. || ⚠️ THE SOURCE GRAPHIC WAS WRONG ON MSFT. It printed 32,488 (+10.1%), which is fiscal 2025 ended Jun 30 2025. Fiscal 2026 ended Jun 30 2026 and the 10-K was filed Jul 29 2026, before the graphic's own stated August 2026 cutoff, so the current figure was available and was not used. The true number is 35,562 (+9.5%), which also lifts MSFT above AAPL to 4th place. Six of the seven figures matched the filings to the dollar; only MSFT did not. || Fiscal calendars are not aligned - NVDA's year ended Jan 25 2026, MSFT's Jun 30 2026, AAPL's Sep 27 2025, and the rest Dec 31 2025 - so this is not a like-for-like comparison of the same twelve months. No board fields, budgets or positions were changed; this is reference information only. || Sep 6, 2026 - MU STRATEGY REVISED. Micron closed at 1,016.59 on Sep 4, through the 1,000 level, +244.5% year-to-date from a Jan 2 base of 295.13 and 19.0% below its 1,255 high. Salee's position - 35.45 shares at an average of 636.998 - is now worth ~36,038 for a gain of ~13,457, up 59.6%. Room unchanged at 7,418.42 on a 30,000 budget; 3.78% of the book. || ⚠️ A FLAW IN MY OWN PLAN, CORRECTED. The standing MU limit order at 750 now sits 26.2% BELOW the market. It would almost certainly never fill, and if it did, a 26% collapse would be a reason to RE-UNDERWRITE the position, not to buy automatically. A rule that cannot fire is not a rule. It has been DELETED and replaced with an evidence-based second rung: 3,418.42 at the Q1 FY2027 print (~mid-December), deployable ONLY if DRAM bit shipments grow double-digit for a SECOND consecutive quarter. Two in a row means the story has genuinely turned from price to volume; one is noise. The 30 Sep rung is unchanged at 4,000 on the same bit-growth test plus gross margin &gt;=80%. Total scheduled 7,418.42 = exactly the room. || ON THE 'SOLD OUT' HEADLINE, WHICH IS THE REASON THE STOCK IS RUNNING - it is weaker evidence than it looks. The claim that all 2027 DRAM and HBM capacity at Samsung, SK hynix and Micron is booked traces to DigiTimes citing 'industry insiders' (Aug 4, 2026), NOT to a Micron disclosure; the same report mentions long-term agreements of up to five years but states nothing about whether these are firm volume commitments, prepayments, or non-binding. Micron's own language in its prepared remarks is narrower: 'We expect tight conditions to persist beyond calendar 2027' - a statement about DURATION, not about being sold out. || ⚠️ THE DISTINCTION THAT MATTERS: being sold out is about ALLOCATION, not PRICE. Fully committed capacity does not stop contracts repricing lower at renewal, and TrendForce has DRAM contract price growth decelerating from +90-95% (1Q26) to +58-63% (2Q26) to +13-18% (3Q26). Micron's own CFO disclosed DRAM bits up 'low-single-digit percentage range' while prices rose in the 'low-60s' - roughly 95% of revenue growth is price. FY2023 remains the precedent: revenue halved from 30,758m to 15,540m and gross margin went NEGATIVE 9.1% on a 5.83bn loss. || CREDIT WHERE DUE - the source post was responsibly balanced, naming cyclicality, a possible supply glut, competition from SK hynix and Samsung, and valuation risk after the rally. Its '+200% from ~315' is an understatement: Jan 2 295.13 to the 1,255 high is +325.2%. || A TRIM IS NOW A LIVE OPTION, RECORDED NOT RECOMMENDED. Analyst fair value spans 361 to 2,200 across 45 analysts - a 6x spread, which IS the cycle uncertainty made visible. Taking something off the table before Sep 30 is a legitimate choice and Salee's to make. Added as a standing HOLD line on the Schedule tab so it is visible rather than forgotten. || Sep 5, 2026 - BOARD BROUGHT TO EXACTLY 1,000,000 at Salee's instruction to follow the standing budget recommendations. Two budgets withdrawn, 5,000 each, both ZERO deployed so no position is stranded and no money moves. Assigned budget 1,010,000 -&gt; 1,000,000, i.e. 100.00% of target for the first time since LHX and FPS were added. Unfilled room 412,694.31 -&gt; 402,694.31. || (1) ZS ZSCALER - budget 5,000 -&gt; None. Flagged as the standing trim candidate on four separate occasions and the reason is now explicit in the data: it is the ONLY LOSS-MAKING name of the three cybersecurity holdings, net margin -1.88% and ROE -2.43%, against PANW and CRWD which are both already deployed and both showing large gains (+94% and +120% respectively). Forward P/E 36.55 with a PEG of 1.39. Group 15 Cybersecurity 25,000 -&gt; 20,000, which is still 2x its deployed 7,675. CONSEQUENCE: ZS was a 5,000 line in TRANCHE 1 of the deployment plan, so Tranche 1 falls 75,697 -&gt; 70,697 and the whole plan 197,311 -&gt; 192,311. The buffer rises correspondingly. || (2) AMPX AMPRIUS TECHNOLOGIES - budget 5,000 -&gt; None. Net margin -43.98% and ROE -44.16% on a 9.89 share price; revenue growth of 172.6% is off a very small base. It was the fifth name in group 8 Defence, Drones &amp; Public Safety, behind PLTR (5,533 deployed), AVAV (3,758), ONDS (2,031) and LHX (5,000 budgeted at Salee's own instruction). Group 8 budget 30,000 -&gt; 25,000. Nothing was deployed and no thesis was ever written for it. || WHY THESE TWO AND NOT OTHERS - every other zero-deployed budget was protected for a stated reason: V and MCD are dated Tranche 1 lines; APP, PL, LUNR, FPS and LHX all carry explicit triggers set within the last three days; IONQ is the board's ONLY quantum name, so cutting it would delete a whole theme rather than trim a duplicate; CAT and AEP are profitable industrials (ROE 56.97% and 10.13%). ZS and AMPX were the only zero-deployed budgets that were BOTH loss-making AND redundant inside an already-funded group. || CONSIDERED AND REJECTED - ONDS was the other candidate on thesis grounds (previously recorded as carrying 'substantial doubt' language and +156% dilution), but it has 2,030.54 deployed, so trimming it would have been a partial cut rather than a clean withdrawal, and its board fields look internally suspect (pm 251.92%, roe 42.95% sit oddly against that thesis). Flagged for the fundamentals job to re-verify rather than acted on with data I do not trust. It remains the next candidate if the target is ever cut below 1,000,000. || Held positions 52 and held cost 597,305.69 UNCHANGED. AI concentration unchanged at the held level - this removes future headroom, not money. Board 181 tickers. || Sep 5, 2026 - THREE APPROVED BOARD ACTIONS EXECUTED TOGETHER at Salee's instruction. || (1) SPACE FUNDED BY TRIMMING TWO ON-HOLD AI-CORE NAMES. ALAB 15,000 -&gt; 7,000 (-8,000) and LITE 20,000 -&gt; 13,000 (-7,000); both budgets remain ABOVE their deployed cost (ALAB 3,805.47, LITE 9,372.74) so no position is stranded. The 15,000 goes to group 7 Space, which rises 10,000 -&gt; 25,000: RKLB unchanged at 10,000 (1,942.58 deployed), PL Planet Labs NEW 10,000, LUNR Intuitive Machines NEW 5,000. RATIONALE - ALAB (fwd P/E 86.95) and LITE (ROE -149.3%) have both been on explicit hold for weeks, so their budgets were dead money; Space carried 1.00% of a 1,005,000 target across six names, too little to express any view. This single move funds the theme AND reduces AI-core budget, addressing the standing concentration problem from both ends. PL is the only name in the group approaching profitability - Q2 FY27 revenue 116.1m +58%, adjusted EBITDA POSITIVE 13.9m, GAAP loss narrowed from -22.6m to -9.4m, cash 865.4m against 448.3m of converts, backlog 814.9m. CAVEAT: PL guided next quarter to 101-105m against 114.3m consensus, a sequential DECLINE - hence the trigger is the ~December print, not now. LUNR revenue tripled to 206.2m with an 1.8bn backlog but debt went 37m -&gt; 481m and shares +44.1% YoY; trigger is IM-3 actually flying. SPCX and ASTS deliberately left unfunded (82x sales; a 231m quarterly loss with debt +492%). || (2) APP BUDGET SET AT 5,000. This corrects a documented discrepancy: the 200k deployment plan has stated since Sep 3 that APP had a 5,000 budget, but the board carried None - the intent was written and never executed. Recorded as an error, not a change of view. NOTHING DEPLOYED - the trigger remains the ~Nov 4 print. WHY APP IS CHEAP, NOW ESTABLISHED: the fall from 745.61 to ~320 is DECELERATION, not fraud. Revenue growth ran 68% -&gt; 66% -&gt; 59% -&gt; 53% -&gt; guided 47%, culminating in a -19.66% day on Aug 6 2026 after the first-ever guidance miss (Q2 revenue 1,924m vs ~1,935m consensus). CEO Foroughi: 'Our pace of meaningful model improvement was lighter than normal during the quarter, and the next step up in model performance landed just after quarter end.' TWO OVERHANGS HAVE RESOLVED IN APP'S FAVOUR - CFO Matt Stumpf stated Aug 5 2026 that 'The SEC has recently advised us that it concluded its inquiry with no recommended action', and CapitalWatch RETRACTED its money-laundering report on Feb 9 2026 citing a 'flawed verification process'. The 2025 Fuzzy Panda/Culper class action remains at motion-to-dismiss, undecided. Short interest only 3.9% of float. Business quality intact: Q2 gross margin 88.3%, net income 1,267m +55%, free cash flow 863m in the quarter. || (3) SIDU REMOVED FROM THE BOARD. Sidus Space had no budget and no position, so nothing is lost. Q2 2026 revenue FELL 54% to 583k while every peer in the group grew; gross margin is NEGATIVE 108%; share count went roughly 18.30m -&gt; 101.21m in twelve months; the company executed a 1-for-100 reverse split in Dec 2023 to regain Nasdaq minimum-bid compliance. It was a row producing noise, not signal. Board 182 -&gt; 181 tickers. || ⚠️ FOUR APP FIELDS ARE WRONG ON THIS BOARD and are flagged for the next fundamentals pass, NOT silently patched here: fpe carried as 24.17 but the true FORWARD P/E is 17.72 (24.65 is the TRAILING multiple); roe carried as 266.44 vs 203.69 sourced; de carried as 1.63 vs 1.11 (3.52bn debt / 3.16bn equity at Jun 30 2026); revG carried as 66.4 which was the Q4 2025 rate - the Q2 2026 YoY is 53%. Recorded rather than corrected because fundamentals belong to the earnings-refresh job. || ⚠️ BUDGET CONSEQUENCE - assigned budget 1,005,000 -&gt; 1,010,000, i.e. 101.0% of the 1,000,000 target. The Space reallocation was budget-NEUTRAL by construction (-15,000 AI core, +15,000 Space); the whole +5,000 is the APP line. ZS remains the standing trim candidate (5,000 budgeted, 0 deployed, weakest of the three cybersecurity names) which would return the board to 1,005,000; a further 5,000 trim is still needed for exactly 1,000,000. Salee has not yet chosen either, so the overage stands and is flagged, not absorbed. || Held positions 52 and held cost 597,305.69 both UNCHANGED - these are budget and roster changes, no money moved. Unfilled room 412,694.31. || Sep 4, 2026 - close. Daily price refresh: 160 of 182 tickers brought to the Friday Sep 4, 2026 close (price, mcapB, pxd; mcapB scaled by each ticker's exact price ratio). METHOD per playbook: stockanalysis.com quote page taken only when stamped "Sep 4, 2026, 4:00 PM EDT" AND its stated previous close tied to the Sep 3 close; partial-session /history/ rows discarded throughout (worst: SITM history close 611.07 above its own high 608.58 - internally impossible; MCD history close below its own low; KTOS/ONDS/RCAT/RBRK/SOUN/WULF/PENG/YUM/BKNG/S rows were low-volume partial captures, quote page used); history-table fallbacks for MMM and FSLR (quote pages intraday-stamped, Sep 4 rows internally consistent); GOOGL prev-close tie via the Sep 3 adjusted close (0.22 dividend adjustment). CONSTRAINT THIS RUN, RECORDED RATHER THAN PAPERED OVER: the session's 200-call WebSearch budget was exhausted mid-run by the 182-ticker fan-out, which also blocks provenance for new second-source URLs, so most late-batch names could not reach Google Finance/marketscreener/ycharts/fool. All 23 moves &gt;=6% were treated per the gate. ELEVEN confirmed against dated independent Sep 4 sources and passed with --allow: AEHR +13.1% (marketscreener), EOSE +10.9% (Google Finance beta 'Closed: Sep 4, 4:00:01 PM GMT-4'), ALAB +9.8%, AXTI +9.7%, POET +8.1%, TSEM +7.9%, NBIS +7.5%, FORM +7.4%, MRVL +7.1%, COHR +6.6% (all Google Finance dated closes), MU +6.1% (GF beta, prev close derived per the after-hours quirk). TWELVE &gt;=6% moves could NOT be second-sourced and were REVERTED to their Sep 3 board values per the stale-beats-wrong rule - each had an internally consistent single-source Sep 4 print (4:00 PM EDT stamp + prev-close tie, most with an exactly agreeing history row) that the next run should confirm and apply: SNDK 1740.00 (+11.9%), COHU 50.72 (+10.3%), SKHY 177.00 (+8.1%), KLAC 185.60 (+7.3%), IREN 44.68 (+7.3%), BE 252.87 (+7.3%), SITM 612.09 (+6.5%), PENG 51.76 (+6.4%), NRG 119.02 (+6.4%), ADBE 266.51 (-6.7%; two Sep-4-dated headlines corroborate a ~7% fall on CEO-succession disappointment but no fetchable second quote), STX 849.28 (+6.3%), HUT 93.55 (+6.2%). Their pxd stays 2026-09-03 so the staleness badges show honestly. UNRESOLVED, left at prior values: POWI/AMBQ/INDI/KEEL/OSS - quote pages pinned to intraday snapshots across repeated cache-busted fetches, no valid Sep 4 history rows; CLPT - no Sep 4 print anywhere reachable (Sep 3 after-hours was +4.6%, so the stale value was deliberately not nudged); FPS/HYLN/AIRJ - stockanalysis never posted their Sep 4 session; VPG - quote page cleanly stam</t>
         </is>
       </c>
     </row>
@@ -6034,10 +6034,10 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>48.63</v>
+        <v>51.76</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>2.4924</v>
+        <v>2.6528</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>40.36</v>

</xml_diff>